<commit_message>
Build QMD ticket auto-router
</commit_message>
<xml_diff>
--- a/backend/tickets.xlsx
+++ b/backend/tickets.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7447ba68eda723c9/Desktop/pracs/QMD Automation/qmd-ticket-router/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{E1A3EE72-1966-4389-B3B1-5AE270C2A839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCAC8BBD-FE45-4A07-BD07-190221EA8ED4}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{E1A3EE72-1966-4389-B3B1-5AE270C2A839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{683D9324-C998-4B22-8AD7-CDE8768312C0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7062F53E-C18B-4751-8B18-97F2A7F44C5A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="56">
   <si>
     <t>Ticket Number</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Queue</t>
   </si>
   <si>
-    <t>INC001</t>
-  </si>
-  <si>
     <t>VPN not working</t>
   </si>
   <si>
@@ -57,9 +54,6 @@
     <t>GenIT</t>
   </si>
   <si>
-    <t>INC002</t>
-  </si>
-  <si>
     <t>Production outage</t>
   </si>
   <si>
@@ -69,9 +63,6 @@
     <t>Research</t>
   </si>
   <si>
-    <t>INC003</t>
-  </si>
-  <si>
     <t>Access request</t>
   </si>
   <si>
@@ -84,9 +75,6 @@
     <t>Access Pod</t>
   </si>
   <si>
-    <t>INC004</t>
-  </si>
-  <si>
     <t>Database failure</t>
   </si>
   <si>
@@ -96,20 +84,122 @@
     <t>Kite</t>
   </si>
   <si>
-    <t>INC005</t>
-  </si>
-  <si>
     <t>Application issue</t>
   </si>
   <si>
     <t>Medical Affairs</t>
+  </si>
+  <si>
+    <t>INC006</t>
+  </si>
+  <si>
+    <t>INC007</t>
+  </si>
+  <si>
+    <t>INC008</t>
+  </si>
+  <si>
+    <t>INC009</t>
+  </si>
+  <si>
+    <t>INC010</t>
+  </si>
+  <si>
+    <t>INC011</t>
+  </si>
+  <si>
+    <t>INC012</t>
+  </si>
+  <si>
+    <t>INC013</t>
+  </si>
+  <si>
+    <t>INC014</t>
+  </si>
+  <si>
+    <t>INC015</t>
+  </si>
+  <si>
+    <t>INC016</t>
+  </si>
+  <si>
+    <t>INC017</t>
+  </si>
+  <si>
+    <t>INC018</t>
+  </si>
+  <si>
+    <t>INC019</t>
+  </si>
+  <si>
+    <t>INC020</t>
+  </si>
+  <si>
+    <t>Gadi</t>
+  </si>
+  <si>
+    <t>citrix</t>
+  </si>
+  <si>
+    <t>G.net</t>
+  </si>
+  <si>
+    <t>Veeva CRM</t>
+  </si>
+  <si>
+    <t>Zoom</t>
+  </si>
+  <si>
+    <t>Password reset</t>
+  </si>
+  <si>
+    <t>Outlook</t>
+  </si>
+  <si>
+    <t>Teams</t>
+  </si>
+  <si>
+    <t>Concur</t>
+  </si>
+  <si>
+    <t>Sap</t>
+  </si>
+  <si>
+    <t>Gadi access request</t>
+  </si>
+  <si>
+    <t>equipmets</t>
+  </si>
+  <si>
+    <t>Lock out</t>
+  </si>
+  <si>
+    <t>maufacturing effect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturing affected </t>
+  </si>
+  <si>
+    <t>INC021</t>
+  </si>
+  <si>
+    <t>INC022</t>
+  </si>
+  <si>
+    <t>INC023</t>
+  </si>
+  <si>
+    <t>INC024</t>
+  </si>
+  <si>
+    <t>INC025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,6 +211,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -468,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6A2BE84-C9A2-4956-BA4D-46EE3833575F}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
@@ -490,90 +586,346 @@
     </row>
     <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>25</v>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>